<commit_message>
[monitoramento 31/08] Controle Semanal com a linha 24-31/08 e Registro de Alteracoes com EC-002 (reexecucao da pausa O4-006) — 21 registros oficiais
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
+++ b/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>CONTROLE SEMANAL AMAZON ADS — WINNET METAIS</t>
   </si>
@@ -95,16 +95,37 @@
   <si>
     <t>Fluxo: preencher os dados do export semanal → revisar Status semanal → registrar Notas → decisões de Ads continuam sendo tomadas pela Skill/Playbook/Parâmetros vigentes.</t>
   </si>
+  <si>
+    <t>17/08/2026–23/08/2026</t>
+  </si>
+  <si>
+    <t>INVESTIGAR</t>
+  </si>
+  <si>
+    <t>Semana forte em atribuição (2 vendas ticket alto via Geral, ACOS 2,5% na Geral). CTR agregado deprimido por anomalia de entrega na SP-PP automática (18,7k impr, CTR 0,07%) → investigar termos na O4. Sem SP-PP, CTR da conta = 0,66% (estável). Bituqueiras: requalificação CONFIRMADA em 25/08 (4 anúncios Em inserção, incl. SP-01 e SP-T). PI SP-01: suspensão MANTIDA em 2ª análise da equipe interna (25/08) — contestação encerrada, permanece pausada; não conta como falha de desempenho.</t>
+  </si>
+  <si>
+    <t>24/08/2026 a 31/08/2026</t>
+  </si>
+  <si>
+    <t>relatorios/amazon/monitoramento-31-08 + ciclos/Monitoramento-31-08.md</t>
+  </si>
+  <si>
+    <t>VIGIA</t>
+  </si>
+  <si>
+    <t>Venda PXP 29/08 sem atribuição até 31/08. Auto L1618-o115/07 encontrada ativa (O4-006 não vigorou); pausada em 31/08. Atribuição de 29–31/08 ainda imatura."Geral DBA: ACOS de janela 83,9% (1 venda) → VIGIA; veredito do lance 0,48 na O5."</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.000%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -148,6 +169,11 @@
       <b/>
       <sz val="9"/>
       <color rgb="FF475569"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -262,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -300,12 +326,12 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -318,12 +344,12 @@
     <xf numFmtId="2" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -336,12 +362,12 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -365,6 +391,21 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -474,11 +515,13 @@
           <a:lstStyle/>
           <a:p>
             <a:r>
+              <a:rPr lang="pt-BR"/>
               <a:t>Tendência semanal de ACOS</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="1"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -542,6 +585,12 @@
                 <c:pt idx="3">
                   <c:v>46251</c:v>
                 </c:pt>
+                <c:pt idx="4">
+                  <c:v>46258</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46265</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -564,10 +613,10 @@
                   <c:v>0.4790067720090293</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>4.2267624347692136E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.46564023302817736</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -730,11 +779,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="1144435120"/>
-        <c:axId val="1144448720"/>
+        <c:axId val="1236001248"/>
+        <c:axId val="1236002880"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1144435120"/>
+        <c:axId val="1236001248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -754,7 +803,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1144448720"/>
+        <c:crossAx val="1236002880"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -762,7 +811,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1144448720"/>
+        <c:axId val="1236002880"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -782,7 +831,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1144435120"/>
+        <c:crossAx val="1236001248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1082,84 +1131,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
     </row>
     <row r="2" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
     </row>
     <row r="3" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
-      <c r="K3" s="37"/>
-      <c r="L3" s="37"/>
-      <c r="M3" s="37"/>
-      <c r="N3" s="37"/>
-      <c r="O3" s="37"/>
-      <c r="P3" s="37"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="42"/>
+      <c r="O3" s="42"/>
+      <c r="P3" s="42"/>
     </row>
     <row r="4" spans="1:16" ht="21.95" customHeight="1">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-      <c r="M4" s="39"/>
-      <c r="N4" s="39"/>
-      <c r="O4" s="39"/>
-      <c r="P4" s="39"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="44"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
+      <c r="N4" s="44"/>
+      <c r="O4" s="44"/>
+      <c r="P4" s="44"/>
     </row>
     <row r="5" spans="1:16" ht="33.950000000000003" customHeight="1">
       <c r="A5" s="3" t="s">
@@ -1408,70 +1457,110 @@
       <c r="P9" s="7"/>
     </row>
     <row r="10" spans="1:16">
-      <c r="A10" s="28"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="11"/>
+      <c r="A10" s="28">
+        <v>46258</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="10">
+        <v>36117</v>
+      </c>
+      <c r="D10" s="10">
+        <v>127</v>
+      </c>
+      <c r="E10" s="33">
+        <v>87.8</v>
+      </c>
+      <c r="F10" s="33">
+        <v>2077.2399999999998</v>
+      </c>
+      <c r="G10" s="11">
+        <v>2</v>
+      </c>
       <c r="H10" s="11"/>
-      <c r="I10" s="12" t="str">
+      <c r="I10" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="13" t="str">
+        <v>23.658769931662867</v>
+      </c>
+      <c r="J10" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="13" t="str">
+        <v>4.2267624347692136E-2</v>
+      </c>
+      <c r="K10" s="13">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L10" s="12" t="str">
+        <v>1.5748031496062992E-2</v>
+      </c>
+      <c r="L10" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M10" s="14" t="str">
+        <v>0.6913385826771653</v>
+      </c>
+      <c r="M10" s="14">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="N10" s="15"/>
-      <c r="O10" s="1"/>
+        <v>3.5163496414430877E-3</v>
+      </c>
+      <c r="N10" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="O10" s="35" t="s">
+        <v>27</v>
+      </c>
       <c r="P10" s="6"/>
     </row>
     <row r="11" spans="1:16">
-      <c r="A11" s="28"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="12" t="str">
+      <c r="A11" s="28">
+        <v>46265</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="38">
+        <v>47770</v>
+      </c>
+      <c r="D11" s="39">
+        <v>197</v>
+      </c>
+      <c r="E11" s="39">
+        <v>156.66</v>
+      </c>
+      <c r="F11" s="37">
+        <v>336.44</v>
+      </c>
+      <c r="G11" s="39">
+        <v>2</v>
+      </c>
+      <c r="H11" s="11">
+        <v>2</v>
+      </c>
+      <c r="I11" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="13" t="str">
+        <v>2.1475807481169413</v>
+      </c>
+      <c r="J11" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="13" t="str">
+        <v>0.46564023302817736</v>
+      </c>
+      <c r="K11" s="13">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L11" s="12" t="str">
+        <v>1.015228426395939E-2</v>
+      </c>
+      <c r="L11" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M11" s="14" t="str">
+        <v>0.79522842639593905</v>
+      </c>
+      <c r="M11" s="14">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="N11" s="15"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="6"/>
+        <v>4.1239271509315471E-3</v>
+      </c>
+      <c r="N11" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="O11" t="s">
+        <v>31</v>
+      </c>
+      <c r="P11" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="28"/>
@@ -1607,7 +1696,7 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="28"/>
-      <c r="B16" s="29"/>
+      <c r="B16" s="36"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
       <c r="E16" s="33"/>
@@ -3091,24 +3180,24 @@
       <c r="P60" s="9"/>
     </row>
     <row r="62" spans="1:16" ht="26.1" customHeight="1">
-      <c r="A62" s="38" t="s">
+      <c r="A62" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="38"/>
-      <c r="C62" s="38"/>
-      <c r="D62" s="38"/>
-      <c r="E62" s="38"/>
-      <c r="F62" s="38"/>
-      <c r="G62" s="38"/>
-      <c r="H62" s="38"/>
-      <c r="I62" s="38"/>
-      <c r="J62" s="38"/>
-      <c r="K62" s="38"/>
-      <c r="L62" s="38"/>
-      <c r="M62" s="38"/>
-      <c r="N62" s="38"/>
-      <c r="O62" s="38"/>
-      <c r="P62" s="38"/>
+      <c r="B62" s="43"/>
+      <c r="C62" s="43"/>
+      <c r="D62" s="43"/>
+      <c r="E62" s="43"/>
+      <c r="F62" s="43"/>
+      <c r="G62" s="43"/>
+      <c r="H62" s="43"/>
+      <c r="I62" s="43"/>
+      <c r="J62" s="43"/>
+      <c r="K62" s="43"/>
+      <c r="L62" s="43"/>
+      <c r="M62" s="43"/>
+      <c r="N62" s="43"/>
+      <c r="O62" s="43"/>
+      <c r="P62" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3144,9 +3233,10 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>